<commit_message>
Step 3 - Venue Editor
</commit_message>
<xml_diff>
--- a/public/data/CineScope_Venue_Import_Template.xlsx
+++ b/public/data/CineScope_Venue_Import_Template.xlsx
@@ -10,7 +10,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Venue Import" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Venue Import'!$A$1:$L$1</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -18,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="9">
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -36,17 +38,23 @@
       <name val="Arial"/>
       <i val="1"/>
       <color rgb="00888888"/>
+      <sz val="8"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <i val="1"/>
+      <color rgb="00666666"/>
       <sz val="10"/>
     </font>
     <font>
       <name val="Arial"/>
       <b val="1"/>
-      <color rgb="002B5797"/>
+      <color rgb="001A365D"/>
       <sz val="14"/>
     </font>
     <font>
       <name val="Arial"/>
-      <sz val="11"/>
+      <sz val="10"/>
     </font>
     <font>
       <name val="Arial"/>
@@ -55,21 +63,12 @@
     </font>
     <font>
       <name val="Arial"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Arial"/>
       <b val="1"/>
-      <color rgb="00CC0000"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <color rgb="00CC0000"/>
+      <color rgb="001A365D"/>
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -78,12 +77,17 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="002B5797"/>
+        <fgColor rgb="001A365D"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFF9E6"/>
+        <fgColor rgb="00E8E8E8"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF3CD"/>
       </patternFill>
     </fill>
   </fills>
@@ -97,34 +101,37 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="00CCCCCC"/>
+        <color rgb="00D0D0D0"/>
       </left>
       <right style="thin">
-        <color rgb="00CCCCCC"/>
+        <color rgb="00D0D0D0"/>
       </right>
       <top style="thin">
-        <color rgb="00CCCCCC"/>
+        <color rgb="00D0D0D0"/>
       </top>
       <bottom style="thin">
-        <color rgb="00CCCCCC"/>
+        <color rgb="00D0D0D0"/>
       </bottom>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -490,20 +497,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L3"/>
+  <dimension ref="A1:L4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="25" customWidth="1" min="1" max="1"/>
-    <col width="25" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
     <col width="18" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
     <col width="16" customWidth="1" min="6" max="6"/>
     <col width="35" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
-    <col width="12" customWidth="1" min="9" max="9"/>
-    <col width="12" customWidth="1" min="10" max="10"/>
-    <col width="10" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
     <col width="30" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
@@ -569,131 +576,190 @@
         </is>
       </c>
     </row>
-    <row r="2">
+    <row r="2" ht="16" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Example Cinema (DELETE THIS ROW)</t>
+          <t>Required</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>EXAMPLE CINEMA</t>
+          <t>Required</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
+          <t>Required</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Required</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Optional</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Required</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>Optional</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>Optional</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>Optional</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>Optional</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>Optional</t>
+        </is>
+      </c>
+      <c r="L2" s="2" t="inlineStr">
+        <is>
+          <t>Optional</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Regal Picturehouse</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>REGAL PICTUREHOUSE</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
           <t>London</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="D3" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>Picturehouse</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>Small Chain</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>123 High Street, Kingsland</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>E8 2PB</t>
+        </is>
+      </c>
+      <c r="I3" s="3" t="inlineStr">
+        <is>
+          <t>51.5484</t>
+        </is>
+      </c>
+      <c r="J3" s="3" t="inlineStr">
+        <is>
+          <t>-0.0755</t>
+        </is>
+      </c>
+      <c r="K3" s="3" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="L3" s="3" t="inlineStr">
+        <is>
+          <t>EXAMPLE ROW - delete before importing</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>The Plaza Cinema</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>THE PLAZA CINEMA</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Galway</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>Ireland</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr"/>
+      <c r="F4" s="3" t="inlineStr">
         <is>
           <t>Independent</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>Independent</t>
-        </is>
-      </c>
-      <c r="G2" s="2" t="inlineStr">
-        <is>
-          <t>123 High Street, London</t>
-        </is>
-      </c>
-      <c r="H2" s="2" t="inlineStr">
-        <is>
-          <t>SW1A 1AA</t>
-        </is>
-      </c>
-      <c r="I2" s="2" t="inlineStr">
-        <is>
-          <t>51.5074</t>
-        </is>
-      </c>
-      <c r="J2" s="2" t="inlineStr">
-        <is>
-          <t>-0.1278</t>
-        </is>
-      </c>
-      <c r="K2" s="2" t="inlineStr">
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>Main Street, Galway</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>H91 XY12</t>
+        </is>
+      </c>
+      <c r="I4" s="3" t="inlineStr"/>
+      <c r="J4" s="3" t="inlineStr"/>
+      <c r="K4" s="3" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
-      <c r="L2" s="2" t="inlineStr">
-        <is>
-          <t>Example row - delete before importing</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>Example Vue Venue (DELETE THIS ROW)</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>VUE EXAMPLE</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>Manchester</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>United Kingdom</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>Vue</t>
-        </is>
-      </c>
-      <c r="F3" s="2" t="inlineStr">
-        <is>
-          <t>Large Chain</t>
-        </is>
-      </c>
-      <c r="G3" s="2" t="inlineStr">
-        <is>
-          <t>456 Oxford Road, Manchester</t>
-        </is>
-      </c>
-      <c r="H3" s="2" t="inlineStr">
-        <is>
-          <t>M1 5QS</t>
-        </is>
-      </c>
-      <c r="I3" s="2" t="inlineStr"/>
-      <c r="J3" s="2" t="inlineStr"/>
-      <c r="K3" s="2" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="L3" s="2" t="inlineStr">
-        <is>
-          <t>Example with no coords - will be geocoded</t>
+      <c r="L4" s="3" t="inlineStr">
+        <is>
+          <t>EXAMPLE ROW - delete before importing</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:L1"/>
   <dataValidations count="3">
-    <dataValidation sqref="D2:D1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Invalid Country" error="Must be &quot;United Kingdom&quot; or &quot;Ireland&quot;" promptTitle="Country" prompt="Select country" type="list">
+    <dataValidation sqref="D3:D1100" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="Invalid Country" error="Please select United Kingdom or Ireland" type="list">
       <formula1>"United Kingdom,Ireland"</formula1>
     </dataValidation>
-    <dataValidation sqref="F2:F1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Invalid Category" error="Must be &quot;Large Chain&quot;, &quot;Small Chain&quot;, or &quot;Independent&quot;" type="list">
+    <dataValidation sqref="F3:F1100" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="Invalid Category" error="Please select Large Chain, Small Chain, or Independent" type="list">
       <formula1>"Large Chain,Small Chain,Independent"</formula1>
     </dataValidation>
-    <dataValidation sqref="K2:K1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid Status" error="Must be &quot;Open&quot; or &quot;Closed&quot;" type="list">
+    <dataValidation sqref="K3:K1100" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid Status" error="Please select Open or Closed" type="list">
       <formula1>"Open,Closed"</formula1>
     </dataValidation>
   </dataValidations>
@@ -704,157 +770,227 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="004472C4"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A23"/>
+  <dimension ref="A1:B23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="80" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="65" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="3" t="inlineStr">
-        <is>
-          <t>CineScope Venue Import Template - Instructions</t>
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>CineScope Venue Import Template</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr"/>
+      <c r="A2" s="5" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="4" t="inlineStr">
-        <is>
-          <t>Fill in the 'Venue Import' sheet with your new venues, then upload this file in CineScope.</t>
+      <c r="A3" s="6" t="inlineStr">
+        <is>
+          <t>How to use:</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr"/>
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>1. Fill in venue details on the 'Venue Import' sheet</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>REQUIRED FIELDS:</t>
+          <t>2. Delete the two yellow example rows before importing</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  - Venue Name: The display name shown on the map</t>
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>3. Required fields: Venue Name, Comscore Name, City, Country, Category</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  - Comscore Name: The name Comscore uses for this cinema (often uppercase)</t>
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>4. If you don't have coordinates, leave Latitude and Longitude blank</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  - City: The city or town</t>
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   - CineScope will attempt to geocode from Address/Postcode</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  - Country: Must be 'United Kingdom' or 'Ireland' (use the dropdown)</t>
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>5. Save the file and upload it in CineScope &gt; Venue Manager &gt; Import</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  - Category: 'Large Chain', 'Small Chain', or 'Independent' (use the dropdown)</t>
-        </is>
-      </c>
+      <c r="A10" s="5" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr"/>
+      <c r="A11" s="6" t="inlineStr">
+        <is>
+          <t>Field Notes:</t>
+        </is>
+      </c>
     </row>
     <row r="12">
-      <c r="A12" s="5" t="inlineStr">
-        <is>
-          <t>OPTIONAL FIELDS:</t>
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <t>Venue Name</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>The display name shown on the CineScope map and in reports</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  - Chain: The chain name (e.g. Odeon, Vue). Leave blank for independents</t>
+      <c r="A13" s="7" t="inlineStr">
+        <is>
+          <t>Comscore Name</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>The EXACT name used in Comscore Grosses By Theatre reports</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  - Address: Full street address - used for automatic coordinate lookup if lat/lng not provided</t>
+      <c r="A14" s="7" t="inlineStr">
+        <is>
+          <t>City</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>City or town name</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  - Postcode: Postcode or Eircode - also used for coordinate lookup</t>
+      <c r="A15" s="7" t="inlineStr">
+        <is>
+          <t>Country</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>Must be 'United Kingdom' or 'Ireland' (dropdown)</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  - Latitude / Longitude: If you know the exact coordinates, enter them here. Otherwise leave blank and CineScope will look them up from the address/postcode</t>
+      <c r="A16" s="7" t="inlineStr">
+        <is>
+          <t>Chain</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>Chain name (e.g. Odeon, Vue). Leave blank for independents</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  - Status: 'Open' (default if left blank) or 'Closed'</t>
+      <c r="A17" s="7" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>Large Chain, Small Chain, or Independent (dropdown)</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  - Notes: Any additional information about the venue</t>
+      <c r="A18" s="7" t="inlineStr">
+        <is>
+          <t>Address</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>Full street address - used for geocoding if lat/lng not provided</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" t="inlineStr"/>
+      <c r="A19" s="7" t="inlineStr">
+        <is>
+          <t>Postcode</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>UK postcode or Irish Eircode - used for geocoding</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="7" t="inlineStr">
         <is>
-          <t>IMPORTANT:</t>
+          <t>Latitude</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>Decimal latitude (e.g. 51.5074). Leave blank to auto-geocode</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  - Delete the two yellow example rows before uploading!</t>
+      <c r="A21" s="7" t="inlineStr">
+        <is>
+          <t>Longitude</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>Decimal longitude (e.g. -0.1278). Leave blank to auto-geocode</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  - Each venue must have either lat/lng OR an address/postcode for map placement</t>
+      <c r="A22" s="7" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>Open (default) or Closed</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  - Duplicate venues (same name + city) will be flagged during import</t>
+      <c r="A23" s="7" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="inlineStr">
+        <is>
+          <t>Any additional notes about the venue</t>
         </is>
       </c>
     </row>

</xml_diff>